<commit_message>
Initial commit with leaderboard and Google Sheets integration
</commit_message>
<xml_diff>
--- a/reports/seeded_teams.xlsx
+++ b/reports/seeded_teams.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="3" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Foosball" sheetId="1" state="visible" r:id="rId1"/>
@@ -859,6 +859,9 @@
           <t>w</t>
         </is>
       </c>
+      <c r="H10" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -892,6 +895,9 @@
           <t>w</t>
         </is>
       </c>
+      <c r="H11" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -920,6 +926,9 @@
       <c r="F12" t="n">
         <v>8</v>
       </c>
+      <c r="H12" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -948,6 +957,9 @@
       <c r="F13" t="n">
         <v>6</v>
       </c>
+      <c r="H13" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -976,6 +988,9 @@
       <c r="F14" t="n">
         <v>6</v>
       </c>
+      <c r="H14" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1070,6 +1085,9 @@
       <c r="F17" t="n">
         <v>4</v>
       </c>
+      <c r="H17" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1098,6 +1116,9 @@
       <c r="F18" t="n">
         <v>1</v>
       </c>
+      <c r="H18" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1126,6 +1147,9 @@
       <c r="F19" t="n">
         <v>8</v>
       </c>
+      <c r="H19" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1154,6 +1178,9 @@
       <c r="F20" t="n">
         <v>2</v>
       </c>
+      <c r="H20" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1182,6 +1209,9 @@
       <c r="F21" t="n">
         <v>3</v>
       </c>
+      <c r="H21" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1210,6 +1240,9 @@
       <c r="F22" t="n">
         <v>2</v>
       </c>
+      <c r="H22" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1238,6 +1271,9 @@
       <c r="F23" t="n">
         <v>4</v>
       </c>
+      <c r="H23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1266,6 +1302,9 @@
       <c r="F24" t="n">
         <v>3</v>
       </c>
+      <c r="H24" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1293,6 +1332,9 @@
       </c>
       <c r="F25" t="n">
         <v>1</v>
+      </c>
+      <c r="H25" t="n">
+        <v>6</v>
       </c>
     </row>
   </sheetData>
@@ -1677,6 +1719,9 @@
       <c r="F10" t="n">
         <v>3</v>
       </c>
+      <c r="H10" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1705,6 +1750,9 @@
       <c r="F11" t="n">
         <v>7</v>
       </c>
+      <c r="H11" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1733,6 +1781,9 @@
       <c r="F12" t="n">
         <v>1</v>
       </c>
+      <c r="H12" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -1761,6 +1812,9 @@
       <c r="F13" t="n">
         <v>2</v>
       </c>
+      <c r="H13" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -1789,6 +1843,9 @@
       <c r="F14" t="n">
         <v>2</v>
       </c>
+      <c r="H14" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -1817,6 +1874,9 @@
       <c r="F15" t="n">
         <v>5</v>
       </c>
+      <c r="H15" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1845,6 +1905,9 @@
       <c r="F16" t="n">
         <v>4</v>
       </c>
+      <c r="H16" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1873,6 +1936,9 @@
       <c r="F17" t="n">
         <v>6</v>
       </c>
+      <c r="H17" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1901,6 +1967,9 @@
       <c r="F18" t="n">
         <v>3</v>
       </c>
+      <c r="H18" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1929,6 +1998,9 @@
       <c r="F19" t="n">
         <v>8</v>
       </c>
+      <c r="H19" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1957,6 +2029,9 @@
       <c r="F20" t="n">
         <v>6</v>
       </c>
+      <c r="H20" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1985,6 +2060,9 @@
       <c r="F21" t="n">
         <v>7</v>
       </c>
+      <c r="H21" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2013,6 +2091,9 @@
       <c r="F22" t="n">
         <v>1</v>
       </c>
+      <c r="H22" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2041,6 +2122,9 @@
       <c r="F23" t="n">
         <v>8</v>
       </c>
+      <c r="H23" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2069,6 +2153,9 @@
       <c r="F24" t="n">
         <v>4</v>
       </c>
+      <c r="H24" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2096,6 +2183,9 @@
       </c>
       <c r="F25" t="n">
         <v>5</v>
+      </c>
+      <c r="H25" t="n">
+        <v>3</v>
       </c>
     </row>
   </sheetData>
@@ -2545,7 +2635,9 @@
         <v>2</v>
       </c>
       <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
+      <c r="H10" t="n">
+        <v>3</v>
+      </c>
       <c r="I10" t="inlineStr"/>
       <c r="J10" t="inlineStr"/>
       <c r="K10" t="inlineStr"/>
@@ -2582,7 +2674,9 @@
         <v>1</v>
       </c>
       <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
+      <c r="H11" t="n">
+        <v>1</v>
+      </c>
       <c r="I11" t="inlineStr"/>
       <c r="J11" t="inlineStr"/>
       <c r="K11" t="inlineStr"/>
@@ -2619,7 +2713,9 @@
         <v>3</v>
       </c>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
+      <c r="H12" t="n">
+        <v>8</v>
+      </c>
       <c r="I12" t="inlineStr"/>
       <c r="J12" t="inlineStr"/>
       <c r="K12" t="inlineStr"/>
@@ -2656,7 +2752,9 @@
         <v>5</v>
       </c>
       <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
+      <c r="H13" t="n">
+        <v>5</v>
+      </c>
       <c r="I13" t="inlineStr"/>
       <c r="J13" t="inlineStr"/>
       <c r="K13" t="inlineStr"/>
@@ -2693,7 +2791,9 @@
         <v>3</v>
       </c>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
+      <c r="H14" t="n">
+        <v>4</v>
+      </c>
       <c r="I14" t="inlineStr"/>
       <c r="J14" t="inlineStr"/>
       <c r="K14" t="inlineStr"/>
@@ -2730,7 +2830,9 @@
         <v>2</v>
       </c>
       <c r="G15" t="inlineStr"/>
-      <c r="H15" t="inlineStr"/>
+      <c r="H15" t="n">
+        <v>7</v>
+      </c>
       <c r="I15" t="inlineStr"/>
       <c r="J15" t="inlineStr"/>
       <c r="K15" t="inlineStr"/>
@@ -2767,7 +2869,9 @@
         <v>7</v>
       </c>
       <c r="G16" t="inlineStr"/>
-      <c r="H16" t="inlineStr"/>
+      <c r="H16" t="n">
+        <v>1</v>
+      </c>
       <c r="I16" t="inlineStr"/>
       <c r="J16" t="inlineStr"/>
       <c r="K16" t="inlineStr"/>
@@ -2804,7 +2908,9 @@
         <v>6</v>
       </c>
       <c r="G17" t="inlineStr"/>
-      <c r="H17" t="inlineStr"/>
+      <c r="H17" t="n">
+        <v>6</v>
+      </c>
       <c r="I17" t="inlineStr"/>
       <c r="J17" t="inlineStr"/>
       <c r="K17" t="inlineStr"/>
@@ -2841,7 +2947,9 @@
         <v>4</v>
       </c>
       <c r="G18" t="inlineStr"/>
-      <c r="H18" t="inlineStr"/>
+      <c r="H18" t="n">
+        <v>2</v>
+      </c>
       <c r="I18" t="inlineStr"/>
       <c r="J18" t="inlineStr"/>
       <c r="K18" t="inlineStr"/>
@@ -2878,7 +2986,9 @@
         <v>1</v>
       </c>
       <c r="G19" t="inlineStr"/>
-      <c r="H19" t="inlineStr"/>
+      <c r="H19" t="n">
+        <v>6</v>
+      </c>
       <c r="I19" t="inlineStr"/>
       <c r="J19" t="inlineStr"/>
       <c r="K19" t="inlineStr"/>
@@ -2915,7 +3025,9 @@
         <v>7</v>
       </c>
       <c r="G20" t="inlineStr"/>
-      <c r="H20" t="inlineStr"/>
+      <c r="H20" t="n">
+        <v>4</v>
+      </c>
       <c r="I20" t="inlineStr"/>
       <c r="J20" t="inlineStr"/>
       <c r="K20" t="inlineStr"/>
@@ -2952,7 +3064,9 @@
         <v>8</v>
       </c>
       <c r="G21" t="inlineStr"/>
-      <c r="H21" t="inlineStr"/>
+      <c r="H21" t="n">
+        <v>5</v>
+      </c>
       <c r="I21" t="inlineStr"/>
       <c r="J21" t="inlineStr"/>
       <c r="K21" t="inlineStr"/>
@@ -2989,7 +3103,9 @@
         <v>5</v>
       </c>
       <c r="G22" t="inlineStr"/>
-      <c r="H22" t="inlineStr"/>
+      <c r="H22" t="n">
+        <v>3</v>
+      </c>
       <c r="I22" t="inlineStr"/>
       <c r="J22" t="inlineStr"/>
       <c r="K22" t="inlineStr"/>
@@ -3026,7 +3142,9 @@
         <v>4</v>
       </c>
       <c r="G23" t="inlineStr"/>
-      <c r="H23" t="inlineStr"/>
+      <c r="H23" t="n">
+        <v>2</v>
+      </c>
       <c r="I23" t="inlineStr"/>
       <c r="J23" t="inlineStr"/>
       <c r="K23" t="inlineStr"/>
@@ -3063,7 +3181,9 @@
         <v>6</v>
       </c>
       <c r="G24" t="inlineStr"/>
-      <c r="H24" t="inlineStr"/>
+      <c r="H24" t="n">
+        <v>8</v>
+      </c>
       <c r="I24" t="inlineStr"/>
       <c r="J24" t="inlineStr"/>
       <c r="K24" t="inlineStr"/>
@@ -3100,7 +3220,9 @@
         <v>8</v>
       </c>
       <c r="G25" t="inlineStr"/>
-      <c r="H25" t="inlineStr"/>
+      <c r="H25" t="n">
+        <v>7</v>
+      </c>
       <c r="I25" t="inlineStr"/>
       <c r="J25" t="inlineStr"/>
       <c r="K25" t="inlineStr"/>
@@ -3675,6 +3797,9 @@
       <c r="E18" t="n">
         <v>13</v>
       </c>
+      <c r="G18" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -3744,6 +3869,9 @@
       <c r="E21" t="n">
         <v>10</v>
       </c>
+      <c r="G21" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -3767,6 +3895,9 @@
       <c r="E22" t="n">
         <v>4</v>
       </c>
+      <c r="G22" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -3790,6 +3921,9 @@
       <c r="E23" t="n">
         <v>7</v>
       </c>
+      <c r="G23" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -3813,6 +3947,9 @@
       <c r="E24" t="n">
         <v>15</v>
       </c>
+      <c r="G24" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -3836,6 +3973,9 @@
       <c r="E25" t="n">
         <v>9</v>
       </c>
+      <c r="G25" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -3859,6 +3999,9 @@
       <c r="E26" t="n">
         <v>7</v>
       </c>
+      <c r="G26" t="n">
+        <v>13</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -3882,6 +4025,9 @@
       <c r="E27" t="n">
         <v>16</v>
       </c>
+      <c r="G27" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -3905,6 +4051,9 @@
       <c r="E28" t="n">
         <v>11</v>
       </c>
+      <c r="G28" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -3928,6 +4077,9 @@
       <c r="E29" t="n">
         <v>15</v>
       </c>
+      <c r="G29" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -3951,6 +4103,9 @@
       <c r="E30" t="n">
         <v>5</v>
       </c>
+      <c r="G30" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -3974,6 +4129,9 @@
       <c r="E31" t="n">
         <v>14</v>
       </c>
+      <c r="G31" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -3997,6 +4155,9 @@
       <c r="E32" t="n">
         <v>12</v>
       </c>
+      <c r="G32" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -4020,6 +4181,9 @@
       <c r="E33" t="n">
         <v>6</v>
       </c>
+      <c r="G33" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -4043,6 +4207,9 @@
       <c r="E34" t="n">
         <v>12</v>
       </c>
+      <c r="G34" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -4066,6 +4233,9 @@
       <c r="E35" t="n">
         <v>2</v>
       </c>
+      <c r="G35" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -4089,6 +4259,9 @@
       <c r="E36" t="n">
         <v>1</v>
       </c>
+      <c r="G36" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -4112,6 +4285,9 @@
       <c r="E37" t="n">
         <v>13</v>
       </c>
+      <c r="G37" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -4135,6 +4311,9 @@
       <c r="E38" t="n">
         <v>8</v>
       </c>
+      <c r="G38" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -4158,6 +4337,9 @@
       <c r="E39" t="n">
         <v>11</v>
       </c>
+      <c r="G39" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -4181,6 +4363,9 @@
       <c r="E40" t="n">
         <v>4</v>
       </c>
+      <c r="G40" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -4204,6 +4389,9 @@
       <c r="E41" t="n">
         <v>5</v>
       </c>
+      <c r="G41" t="n">
+        <v>14</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -4227,6 +4415,9 @@
       <c r="E42" t="n">
         <v>14</v>
       </c>
+      <c r="G42" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -4250,6 +4441,9 @@
       <c r="E43" t="n">
         <v>1</v>
       </c>
+      <c r="G43" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -4273,6 +4467,9 @@
       <c r="E44" t="n">
         <v>6</v>
       </c>
+      <c r="G44" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -4296,6 +4493,9 @@
       <c r="E45" t="n">
         <v>9</v>
       </c>
+      <c r="G45" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -4319,6 +4519,9 @@
       <c r="E46" t="n">
         <v>3</v>
       </c>
+      <c r="G46" t="n">
+        <v>15</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -4342,6 +4545,9 @@
       <c r="E47" t="n">
         <v>10</v>
       </c>
+      <c r="G47" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -4365,6 +4571,9 @@
       <c r="E48" t="n">
         <v>8</v>
       </c>
+      <c r="G48" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -4387,6 +4596,9 @@
       </c>
       <c r="E49" t="n">
         <v>2</v>
+      </c>
+      <c r="G49" t="n">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -4771,6 +4983,9 @@
       <c r="F10" t="n">
         <v>1</v>
       </c>
+      <c r="H10" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -4799,6 +5014,9 @@
       <c r="F11" t="n">
         <v>7</v>
       </c>
+      <c r="H11" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -4827,6 +5045,9 @@
       <c r="F12" t="n">
         <v>8</v>
       </c>
+      <c r="H12" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -4855,6 +5076,9 @@
       <c r="F13" t="n">
         <v>3</v>
       </c>
+      <c r="H13" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -4883,6 +5107,9 @@
       <c r="F14" t="n">
         <v>1</v>
       </c>
+      <c r="H14" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -4911,6 +5138,9 @@
       <c r="F15" t="n">
         <v>7</v>
       </c>
+      <c r="H15" t="n">
+        <v>6</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -4939,6 +5169,9 @@
       <c r="F16" t="n">
         <v>3</v>
       </c>
+      <c r="H16" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -4967,6 +5200,9 @@
       <c r="F17" t="n">
         <v>5</v>
       </c>
+      <c r="H17" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -4995,6 +5231,9 @@
       <c r="F18" t="n">
         <v>6</v>
       </c>
+      <c r="H18" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -5023,6 +5262,9 @@
       <c r="F19" t="n">
         <v>4</v>
       </c>
+      <c r="H19" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -5051,6 +5293,9 @@
       <c r="F20" t="n">
         <v>2</v>
       </c>
+      <c r="H20" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -5079,6 +5324,9 @@
       <c r="F21" t="n">
         <v>5</v>
       </c>
+      <c r="H21" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -5107,6 +5355,9 @@
       <c r="F22" t="n">
         <v>4</v>
       </c>
+      <c r="H22" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -5135,6 +5386,9 @@
       <c r="F23" t="n">
         <v>2</v>
       </c>
+      <c r="H23" t="n">
+        <v>7</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -5163,6 +5417,9 @@
       <c r="F24" t="n">
         <v>6</v>
       </c>
+      <c r="H24" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -5190,6 +5447,9 @@
       </c>
       <c r="F25" t="n">
         <v>8</v>
+      </c>
+      <c r="H25" t="n">
+        <v>6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>